<commit_message>
fix: repair claims worksheet dimensions
</commit_message>
<xml_diff>
--- a/public/retailer-deduction-triage-worksheet.xlsx
+++ b/public/retailer-deduction-triage-worksheet.xlsx
@@ -145,7 +145,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O41"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="4" width="18" customWidth="1"/>
@@ -2761,7 +2761,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J17"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -3661,7 +3661,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>

</xml_diff>

<commit_message>
fix: narrow claims worksheet code timing
</commit_message>
<xml_diff>
--- a/public/retailer-deduction-triage-worksheet.xlsx
+++ b/public/retailer-deduction-triage-worksheet.xlsx
@@ -111,7 +111,7 @@
       </c>
       <c r="B3" t="inlineStr" s="2">
         <is>
-          <t>Pick the deduction type, enter delivery and claim dates, and let the matrix formulas fill the baseline verdict, evidence, Code check, and neutral query.</t>
+          <t>Enter a deduction type ID or visible label from the Matrix tab, add dates, and let the formulas fill the baseline verdict, evidence, Code check, and neutral query.</t>
         </is>
       </c>
     </row>
@@ -123,7 +123,7 @@
       </c>
       <c r="B4" t="inlineStr" s="2">
         <is>
-          <t>Shortfall and damaged-goods lines flag when the claim date is more than 30 days after delivery.</t>
+          <t>Fresh produce shortfall and damaged-goods lines flag when the claim date is more than 30 days after delivery.</t>
         </is>
       </c>
     </row>
@@ -145,17 +145,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:P41"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="11" width="34" customWidth="1"/>
-    <col min="12" max="12" width="32" customWidth="1"/>
-    <col min="13" max="15" width="16" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="12" width="34" customWidth="1"/>
+    <col min="13" max="13" width="36" customWidth="1"/>
+    <col min="14" max="16" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -181,55 +182,60 @@
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
+          <t>Fresh produce? (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
           <t>Deduction type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
+      <c r="G1" t="inlineStr" s="1">
         <is>
           <t>Reason note</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="K1" t="inlineStr" s="1">
         <is>
           <t>Code check</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="L1" t="inlineStr" s="1">
         <is>
           <t>Neutral query</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
+      <c r="M1" t="inlineStr" s="1">
         <is>
           <t>Gap</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="1">
+      <c r="N1" t="inlineStr" s="1">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr" s="1">
+      <c r="O1" t="inlineStr" s="1">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr" s="1">
+      <c r="P1" t="inlineStr" s="1">
         <is>
           <t>Status</t>
         </is>
@@ -266,33 +272,38 @@
           <t/>
         </is>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2" s="3">
         <v>0</v>
       </c>
-      <c r="H2">
-        <f>IF($E2="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E2,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I2" s="2">
-        <f>IF($E2="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E2,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I2">
+        <f>IF($F2="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F2,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F2,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J2" s="2">
-        <f>IF($E2="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E2,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F2="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F2,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F2,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K2" s="2">
-        <f>IF($E2="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E2,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F2="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F2,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F2,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L2" s="2">
-        <f>IF(AND(OR($E2="shortfall",$E2="damaged-goods"),$C2&lt;&gt;"",$D2&lt;&gt;"",$D2-$C2&gt;30),"Claim raised more than 30 days after delivery.",IF($H2="missing proof","Await line-level proof from the retailer.",IF($H2="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H2="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M2">
-        <f>IF($E2="","",IF(AND(OR($E2="shortfall",$E2="damaged-goods"),$C2&lt;&gt;"",$D2&lt;&gt;"",$D2-$C2&gt;30),"High",IF(OR($H2="Code risk",$G2&gt;=5000),"High",IF(OR($H2="missing proof",$G2&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F2="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F2,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F2,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M2" s="2">
+        <f>IF(AND(AND(OR($F2="shortfall",$F2="damaged-goods",$F2="Shortfall / short-delivery",$F2="Damaged goods"),AND($C2&lt;&gt;"",$D2&lt;&gt;"",$D2-$C2&gt;30)),OR(UPPER($E2)="Y",UPPER($E2)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F2="shortfall",$F2="damaged-goods",$F2="Shortfall / short-delivery",$F2="Damaged goods"),AND($C2&lt;&gt;"",$D2&lt;&gt;"",$D2-$C2&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I2="missing proof","Await line-level proof from the retailer.",IF($I2="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I2="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N2">
+        <f>IF($F2="","",IF(AND(AND(OR($F2="shortfall",$F2="damaged-goods",$F2="Shortfall / short-delivery",$F2="Damaged goods"),AND($C2&lt;&gt;"",$D2&lt;&gt;"",$D2-$C2&gt;30)),OR(UPPER($E2)="Y",UPPER($E2)="YES")),"High",IF(OR($I2="Code risk",$H2&gt;=5000),"High",IF(OR($I2="missing proof",$H2&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -329,33 +340,38 @@
           <t/>
         </is>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" s="3">
         <v>0</v>
       </c>
-      <c r="H3">
-        <f>IF($E3="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E3,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I3" s="2">
-        <f>IF($E3="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E3,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I3">
+        <f>IF($F3="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F3,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F3,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J3" s="2">
-        <f>IF($E3="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E3,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F3="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F3,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F3,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K3" s="2">
-        <f>IF($E3="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E3,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F3="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F3,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F3,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L3" s="2">
-        <f>IF(AND(OR($E3="shortfall",$E3="damaged-goods"),$C3&lt;&gt;"",$D3&lt;&gt;"",$D3-$C3&gt;30),"Claim raised more than 30 days after delivery.",IF($H3="missing proof","Await line-level proof from the retailer.",IF($H3="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H3="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M3">
-        <f>IF($E3="","",IF(AND(OR($E3="shortfall",$E3="damaged-goods"),$C3&lt;&gt;"",$D3&lt;&gt;"",$D3-$C3&gt;30),"High",IF(OR($H3="Code risk",$G3&gt;=5000),"High",IF(OR($H3="missing proof",$G3&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F3="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F3,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F3,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M3" s="2">
+        <f>IF(AND(AND(OR($F3="shortfall",$F3="damaged-goods",$F3="Shortfall / short-delivery",$F3="Damaged goods"),AND($C3&lt;&gt;"",$D3&lt;&gt;"",$D3-$C3&gt;30)),OR(UPPER($E3)="Y",UPPER($E3)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F3="shortfall",$F3="damaged-goods",$F3="Shortfall / short-delivery",$F3="Damaged goods"),AND($C3&lt;&gt;"",$D3&lt;&gt;"",$D3-$C3&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I3="missing proof","Await line-level proof from the retailer.",IF($I3="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I3="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N3">
+        <f>IF($F3="","",IF(AND(AND(OR($F3="shortfall",$F3="damaged-goods",$F3="Shortfall / short-delivery",$F3="Damaged goods"),AND($C3&lt;&gt;"",$D3&lt;&gt;"",$D3-$C3&gt;30)),OR(UPPER($E3)="Y",UPPER($E3)="YES")),"High",IF(OR($I3="Code risk",$H3&gt;=5000),"High",IF(OR($I3="missing proof",$H3&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -392,33 +408,38 @@
           <t/>
         </is>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H4" s="3">
         <v>0</v>
       </c>
-      <c r="H4">
-        <f>IF($E4="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E4,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I4" s="2">
-        <f>IF($E4="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E4,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I4">
+        <f>IF($F4="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F4,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F4,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J4" s="2">
-        <f>IF($E4="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E4,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F4="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F4,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F4,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K4" s="2">
-        <f>IF($E4="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E4,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F4="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F4,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F4,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L4" s="2">
-        <f>IF(AND(OR($E4="shortfall",$E4="damaged-goods"),$C4&lt;&gt;"",$D4&lt;&gt;"",$D4-$C4&gt;30),"Claim raised more than 30 days after delivery.",IF($H4="missing proof","Await line-level proof from the retailer.",IF($H4="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H4="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M4">
-        <f>IF($E4="","",IF(AND(OR($E4="shortfall",$E4="damaged-goods"),$C4&lt;&gt;"",$D4&lt;&gt;"",$D4-$C4&gt;30),"High",IF(OR($H4="Code risk",$G4&gt;=5000),"High",IF(OR($H4="missing proof",$G4&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F4="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F4,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F4,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M4" s="2">
+        <f>IF(AND(AND(OR($F4="shortfall",$F4="damaged-goods",$F4="Shortfall / short-delivery",$F4="Damaged goods"),AND($C4&lt;&gt;"",$D4&lt;&gt;"",$D4-$C4&gt;30)),OR(UPPER($E4)="Y",UPPER($E4)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F4="shortfall",$F4="damaged-goods",$F4="Shortfall / short-delivery",$F4="Damaged goods"),AND($C4&lt;&gt;"",$D4&lt;&gt;"",$D4-$C4&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I4="missing proof","Await line-level proof from the retailer.",IF($I4="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I4="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N4">
+        <f>IF($F4="","",IF(AND(AND(OR($F4="shortfall",$F4="damaged-goods",$F4="Shortfall / short-delivery",$F4="Damaged goods"),AND($C4&lt;&gt;"",$D4&lt;&gt;"",$D4-$C4&gt;30)),OR(UPPER($E4)="Y",UPPER($E4)="YES")),"High",IF(OR($I4="Code risk",$H4&gt;=5000),"High",IF(OR($I4="missing proof",$H4&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -455,33 +476,38 @@
           <t/>
         </is>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H5" s="3">
         <v>0</v>
       </c>
-      <c r="H5">
-        <f>IF($E5="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E5,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I5" s="2">
-        <f>IF($E5="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E5,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I5">
+        <f>IF($F5="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F5,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F5,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J5" s="2">
-        <f>IF($E5="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E5,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F5="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F5,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F5,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K5" s="2">
-        <f>IF($E5="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E5,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F5="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F5,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F5,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L5" s="2">
-        <f>IF(AND(OR($E5="shortfall",$E5="damaged-goods"),$C5&lt;&gt;"",$D5&lt;&gt;"",$D5-$C5&gt;30),"Claim raised more than 30 days after delivery.",IF($H5="missing proof","Await line-level proof from the retailer.",IF($H5="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H5="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M5">
-        <f>IF($E5="","",IF(AND(OR($E5="shortfall",$E5="damaged-goods"),$C5&lt;&gt;"",$D5&lt;&gt;"",$D5-$C5&gt;30),"High",IF(OR($H5="Code risk",$G5&gt;=5000),"High",IF(OR($H5="missing proof",$G5&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F5="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F5,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F5,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M5" s="2">
+        <f>IF(AND(AND(OR($F5="shortfall",$F5="damaged-goods",$F5="Shortfall / short-delivery",$F5="Damaged goods"),AND($C5&lt;&gt;"",$D5&lt;&gt;"",$D5-$C5&gt;30)),OR(UPPER($E5)="Y",UPPER($E5)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F5="shortfall",$F5="damaged-goods",$F5="Shortfall / short-delivery",$F5="Damaged goods"),AND($C5&lt;&gt;"",$D5&lt;&gt;"",$D5-$C5&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I5="missing proof","Await line-level proof from the retailer.",IF($I5="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I5="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N5">
+        <f>IF($F5="","",IF(AND(AND(OR($F5="shortfall",$F5="damaged-goods",$F5="Shortfall / short-delivery",$F5="Damaged goods"),AND($C5&lt;&gt;"",$D5&lt;&gt;"",$D5-$C5&gt;30)),OR(UPPER($E5)="Y",UPPER($E5)="YES")),"High",IF(OR($I5="Code risk",$H5&gt;=5000),"High",IF(OR($I5="missing proof",$H5&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -518,33 +544,38 @@
           <t/>
         </is>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" s="3">
         <v>0</v>
       </c>
-      <c r="H6">
-        <f>IF($E6="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E6,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I6" s="2">
-        <f>IF($E6="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E6,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I6">
+        <f>IF($F6="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F6,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F6,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J6" s="2">
-        <f>IF($E6="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E6,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F6="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F6,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F6,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K6" s="2">
-        <f>IF($E6="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E6,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F6="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F6,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F6,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L6" s="2">
-        <f>IF(AND(OR($E6="shortfall",$E6="damaged-goods"),$C6&lt;&gt;"",$D6&lt;&gt;"",$D6-$C6&gt;30),"Claim raised more than 30 days after delivery.",IF($H6="missing proof","Await line-level proof from the retailer.",IF($H6="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H6="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M6">
-        <f>IF($E6="","",IF(AND(OR($E6="shortfall",$E6="damaged-goods"),$C6&lt;&gt;"",$D6&lt;&gt;"",$D6-$C6&gt;30),"High",IF(OR($H6="Code risk",$G6&gt;=5000),"High",IF(OR($H6="missing proof",$G6&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F6="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F6,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F6,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M6" s="2">
+        <f>IF(AND(AND(OR($F6="shortfall",$F6="damaged-goods",$F6="Shortfall / short-delivery",$F6="Damaged goods"),AND($C6&lt;&gt;"",$D6&lt;&gt;"",$D6-$C6&gt;30)),OR(UPPER($E6)="Y",UPPER($E6)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F6="shortfall",$F6="damaged-goods",$F6="Shortfall / short-delivery",$F6="Damaged goods"),AND($C6&lt;&gt;"",$D6&lt;&gt;"",$D6-$C6&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I6="missing proof","Await line-level proof from the retailer.",IF($I6="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I6="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N6">
+        <f>IF($F6="","",IF(AND(AND(OR($F6="shortfall",$F6="damaged-goods",$F6="Shortfall / short-delivery",$F6="Damaged goods"),AND($C6&lt;&gt;"",$D6&lt;&gt;"",$D6-$C6&gt;30)),OR(UPPER($E6)="Y",UPPER($E6)="YES")),"High",IF(OR($I6="Code risk",$H6&gt;=5000),"High",IF(OR($I6="missing proof",$H6&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -581,33 +612,38 @@
           <t/>
         </is>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H7" s="3">
         <v>0</v>
       </c>
-      <c r="H7">
-        <f>IF($E7="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E7,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I7" s="2">
-        <f>IF($E7="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E7,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I7">
+        <f>IF($F7="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F7,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F7,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J7" s="2">
-        <f>IF($E7="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E7,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F7="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F7,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F7,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K7" s="2">
-        <f>IF($E7="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E7,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F7="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F7,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F7,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L7" s="2">
-        <f>IF(AND(OR($E7="shortfall",$E7="damaged-goods"),$C7&lt;&gt;"",$D7&lt;&gt;"",$D7-$C7&gt;30),"Claim raised more than 30 days after delivery.",IF($H7="missing proof","Await line-level proof from the retailer.",IF($H7="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H7="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M7">
-        <f>IF($E7="","",IF(AND(OR($E7="shortfall",$E7="damaged-goods"),$C7&lt;&gt;"",$D7&lt;&gt;"",$D7-$C7&gt;30),"High",IF(OR($H7="Code risk",$G7&gt;=5000),"High",IF(OR($H7="missing proof",$G7&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F7="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F7,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F7,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M7" s="2">
+        <f>IF(AND(AND(OR($F7="shortfall",$F7="damaged-goods",$F7="Shortfall / short-delivery",$F7="Damaged goods"),AND($C7&lt;&gt;"",$D7&lt;&gt;"",$D7-$C7&gt;30)),OR(UPPER($E7)="Y",UPPER($E7)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F7="shortfall",$F7="damaged-goods",$F7="Shortfall / short-delivery",$F7="Damaged goods"),AND($C7&lt;&gt;"",$D7&lt;&gt;"",$D7-$C7&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I7="missing proof","Await line-level proof from the retailer.",IF($I7="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I7="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N7">
+        <f>IF($F7="","",IF(AND(AND(OR($F7="shortfall",$F7="damaged-goods",$F7="Shortfall / short-delivery",$F7="Damaged goods"),AND($C7&lt;&gt;"",$D7&lt;&gt;"",$D7-$C7&gt;30)),OR(UPPER($E7)="Y",UPPER($E7)="YES")),"High",IF(OR($I7="Code risk",$H7&gt;=5000),"High",IF(OR($I7="missing proof",$H7&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -644,33 +680,38 @@
           <t/>
         </is>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H8" s="3">
         <v>0</v>
       </c>
-      <c r="H8">
-        <f>IF($E8="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E8,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I8" s="2">
-        <f>IF($E8="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E8,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I8">
+        <f>IF($F8="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F8,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F8,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J8" s="2">
-        <f>IF($E8="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E8,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F8="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F8,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F8,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K8" s="2">
-        <f>IF($E8="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E8,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F8="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F8,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F8,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L8" s="2">
-        <f>IF(AND(OR($E8="shortfall",$E8="damaged-goods"),$C8&lt;&gt;"",$D8&lt;&gt;"",$D8-$C8&gt;30),"Claim raised more than 30 days after delivery.",IF($H8="missing proof","Await line-level proof from the retailer.",IF($H8="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H8="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M8">
-        <f>IF($E8="","",IF(AND(OR($E8="shortfall",$E8="damaged-goods"),$C8&lt;&gt;"",$D8&lt;&gt;"",$D8-$C8&gt;30),"High",IF(OR($H8="Code risk",$G8&gt;=5000),"High",IF(OR($H8="missing proof",$G8&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F8="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F8,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F8,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M8" s="2">
+        <f>IF(AND(AND(OR($F8="shortfall",$F8="damaged-goods",$F8="Shortfall / short-delivery",$F8="Damaged goods"),AND($C8&lt;&gt;"",$D8&lt;&gt;"",$D8-$C8&gt;30)),OR(UPPER($E8)="Y",UPPER($E8)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F8="shortfall",$F8="damaged-goods",$F8="Shortfall / short-delivery",$F8="Damaged goods"),AND($C8&lt;&gt;"",$D8&lt;&gt;"",$D8-$C8&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I8="missing proof","Await line-level proof from the retailer.",IF($I8="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I8="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N8">
+        <f>IF($F8="","",IF(AND(AND(OR($F8="shortfall",$F8="damaged-goods",$F8="Shortfall / short-delivery",$F8="Damaged goods"),AND($C8&lt;&gt;"",$D8&lt;&gt;"",$D8-$C8&gt;30)),OR(UPPER($E8)="Y",UPPER($E8)="YES")),"High",IF(OR($I8="Code risk",$H8&gt;=5000),"High",IF(OR($I8="missing proof",$H8&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -707,33 +748,38 @@
           <t/>
         </is>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H9" s="3">
         <v>0</v>
       </c>
-      <c r="H9">
-        <f>IF($E9="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E9,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I9" s="2">
-        <f>IF($E9="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E9,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I9">
+        <f>IF($F9="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F9,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F9,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J9" s="2">
-        <f>IF($E9="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E9,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F9="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F9,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F9,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K9" s="2">
-        <f>IF($E9="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E9,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F9="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F9,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F9,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L9" s="2">
-        <f>IF(AND(OR($E9="shortfall",$E9="damaged-goods"),$C9&lt;&gt;"",$D9&lt;&gt;"",$D9-$C9&gt;30),"Claim raised more than 30 days after delivery.",IF($H9="missing proof","Await line-level proof from the retailer.",IF($H9="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H9="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M9">
-        <f>IF($E9="","",IF(AND(OR($E9="shortfall",$E9="damaged-goods"),$C9&lt;&gt;"",$D9&lt;&gt;"",$D9-$C9&gt;30),"High",IF(OR($H9="Code risk",$G9&gt;=5000),"High",IF(OR($H9="missing proof",$G9&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F9="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F9,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F9,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M9" s="2">
+        <f>IF(AND(AND(OR($F9="shortfall",$F9="damaged-goods",$F9="Shortfall / short-delivery",$F9="Damaged goods"),AND($C9&lt;&gt;"",$D9&lt;&gt;"",$D9-$C9&gt;30)),OR(UPPER($E9)="Y",UPPER($E9)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F9="shortfall",$F9="damaged-goods",$F9="Shortfall / short-delivery",$F9="Damaged goods"),AND($C9&lt;&gt;"",$D9&lt;&gt;"",$D9-$C9&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I9="missing proof","Await line-level proof from the retailer.",IF($I9="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I9="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N9">
+        <f>IF($F9="","",IF(AND(AND(OR($F9="shortfall",$F9="damaged-goods",$F9="Shortfall / short-delivery",$F9="Damaged goods"),AND($C9&lt;&gt;"",$D9&lt;&gt;"",$D9-$C9&gt;30)),OR(UPPER($E9)="Y",UPPER($E9)="YES")),"High",IF(OR($I9="Code risk",$H9&gt;=5000),"High",IF(OR($I9="missing proof",$H9&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -770,33 +816,38 @@
           <t/>
         </is>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H10" s="3">
         <v>0</v>
       </c>
-      <c r="H10">
-        <f>IF($E10="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E10,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I10" s="2">
-        <f>IF($E10="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E10,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I10">
+        <f>IF($F10="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F10,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F10,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J10" s="2">
-        <f>IF($E10="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E10,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F10="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F10,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F10,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K10" s="2">
-        <f>IF($E10="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E10,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F10="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F10,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F10,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L10" s="2">
-        <f>IF(AND(OR($E10="shortfall",$E10="damaged-goods"),$C10&lt;&gt;"",$D10&lt;&gt;"",$D10-$C10&gt;30),"Claim raised more than 30 days after delivery.",IF($H10="missing proof","Await line-level proof from the retailer.",IF($H10="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H10="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M10">
-        <f>IF($E10="","",IF(AND(OR($E10="shortfall",$E10="damaged-goods"),$C10&lt;&gt;"",$D10&lt;&gt;"",$D10-$C10&gt;30),"High",IF(OR($H10="Code risk",$G10&gt;=5000),"High",IF(OR($H10="missing proof",$G10&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F10="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F10,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F10,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M10" s="2">
+        <f>IF(AND(AND(OR($F10="shortfall",$F10="damaged-goods",$F10="Shortfall / short-delivery",$F10="Damaged goods"),AND($C10&lt;&gt;"",$D10&lt;&gt;"",$D10-$C10&gt;30)),OR(UPPER($E10)="Y",UPPER($E10)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F10="shortfall",$F10="damaged-goods",$F10="Shortfall / short-delivery",$F10="Damaged goods"),AND($C10&lt;&gt;"",$D10&lt;&gt;"",$D10-$C10&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I10="missing proof","Await line-level proof from the retailer.",IF($I10="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I10="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N10">
+        <f>IF($F10="","",IF(AND(AND(OR($F10="shortfall",$F10="damaged-goods",$F10="Shortfall / short-delivery",$F10="Damaged goods"),AND($C10&lt;&gt;"",$D10&lt;&gt;"",$D10-$C10&gt;30)),OR(UPPER($E10)="Y",UPPER($E10)="YES")),"High",IF(OR($I10="Code risk",$H10&gt;=5000),"High",IF(OR($I10="missing proof",$H10&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -833,33 +884,38 @@
           <t/>
         </is>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H11" s="3">
         <v>0</v>
       </c>
-      <c r="H11">
-        <f>IF($E11="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E11,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I11" s="2">
-        <f>IF($E11="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E11,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I11">
+        <f>IF($F11="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F11,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F11,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J11" s="2">
-        <f>IF($E11="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E11,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F11="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F11,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F11,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K11" s="2">
-        <f>IF($E11="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E11,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F11="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F11,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F11,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L11" s="2">
-        <f>IF(AND(OR($E11="shortfall",$E11="damaged-goods"),$C11&lt;&gt;"",$D11&lt;&gt;"",$D11-$C11&gt;30),"Claim raised more than 30 days after delivery.",IF($H11="missing proof","Await line-level proof from the retailer.",IF($H11="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H11="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M11">
-        <f>IF($E11="","",IF(AND(OR($E11="shortfall",$E11="damaged-goods"),$C11&lt;&gt;"",$D11&lt;&gt;"",$D11-$C11&gt;30),"High",IF(OR($H11="Code risk",$G11&gt;=5000),"High",IF(OR($H11="missing proof",$G11&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F11="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F11,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F11,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M11" s="2">
+        <f>IF(AND(AND(OR($F11="shortfall",$F11="damaged-goods",$F11="Shortfall / short-delivery",$F11="Damaged goods"),AND($C11&lt;&gt;"",$D11&lt;&gt;"",$D11-$C11&gt;30)),OR(UPPER($E11)="Y",UPPER($E11)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F11="shortfall",$F11="damaged-goods",$F11="Shortfall / short-delivery",$F11="Damaged goods"),AND($C11&lt;&gt;"",$D11&lt;&gt;"",$D11-$C11&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I11="missing proof","Await line-level proof from the retailer.",IF($I11="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I11="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N11">
+        <f>IF($F11="","",IF(AND(AND(OR($F11="shortfall",$F11="damaged-goods",$F11="Shortfall / short-delivery",$F11="Damaged goods"),AND($C11&lt;&gt;"",$D11&lt;&gt;"",$D11-$C11&gt;30)),OR(UPPER($E11)="Y",UPPER($E11)="YES")),"High",IF(OR($I11="Code risk",$H11&gt;=5000),"High",IF(OR($I11="missing proof",$H11&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -896,33 +952,38 @@
           <t/>
         </is>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H12" s="3">
         <v>0</v>
       </c>
-      <c r="H12">
-        <f>IF($E12="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E12,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I12" s="2">
-        <f>IF($E12="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E12,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I12">
+        <f>IF($F12="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F12,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F12,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J12" s="2">
-        <f>IF($E12="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E12,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F12="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F12,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F12,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K12" s="2">
-        <f>IF($E12="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E12,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F12="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F12,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F12,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L12" s="2">
-        <f>IF(AND(OR($E12="shortfall",$E12="damaged-goods"),$C12&lt;&gt;"",$D12&lt;&gt;"",$D12-$C12&gt;30),"Claim raised more than 30 days after delivery.",IF($H12="missing proof","Await line-level proof from the retailer.",IF($H12="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H12="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M12">
-        <f>IF($E12="","",IF(AND(OR($E12="shortfall",$E12="damaged-goods"),$C12&lt;&gt;"",$D12&lt;&gt;"",$D12-$C12&gt;30),"High",IF(OR($H12="Code risk",$G12&gt;=5000),"High",IF(OR($H12="missing proof",$G12&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F12="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F12,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F12,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M12" s="2">
+        <f>IF(AND(AND(OR($F12="shortfall",$F12="damaged-goods",$F12="Shortfall / short-delivery",$F12="Damaged goods"),AND($C12&lt;&gt;"",$D12&lt;&gt;"",$D12-$C12&gt;30)),OR(UPPER($E12)="Y",UPPER($E12)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F12="shortfall",$F12="damaged-goods",$F12="Shortfall / short-delivery",$F12="Damaged goods"),AND($C12&lt;&gt;"",$D12&lt;&gt;"",$D12-$C12&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I12="missing proof","Await line-level proof from the retailer.",IF($I12="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I12="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N12">
+        <f>IF($F12="","",IF(AND(AND(OR($F12="shortfall",$F12="damaged-goods",$F12="Shortfall / short-delivery",$F12="Damaged goods"),AND($C12&lt;&gt;"",$D12&lt;&gt;"",$D12-$C12&gt;30)),OR(UPPER($E12)="Y",UPPER($E12)="YES")),"High",IF(OR($I12="Code risk",$H12&gt;=5000),"High",IF(OR($I12="missing proof",$H12&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -959,33 +1020,38 @@
           <t/>
         </is>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H13" s="3">
         <v>0</v>
       </c>
-      <c r="H13">
-        <f>IF($E13="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E13,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I13" s="2">
-        <f>IF($E13="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E13,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I13">
+        <f>IF($F13="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F13,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F13,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J13" s="2">
-        <f>IF($E13="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E13,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F13="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F13,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F13,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K13" s="2">
-        <f>IF($E13="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E13,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F13="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F13,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F13,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L13" s="2">
-        <f>IF(AND(OR($E13="shortfall",$E13="damaged-goods"),$C13&lt;&gt;"",$D13&lt;&gt;"",$D13-$C13&gt;30),"Claim raised more than 30 days after delivery.",IF($H13="missing proof","Await line-level proof from the retailer.",IF($H13="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H13="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M13">
-        <f>IF($E13="","",IF(AND(OR($E13="shortfall",$E13="damaged-goods"),$C13&lt;&gt;"",$D13&lt;&gt;"",$D13-$C13&gt;30),"High",IF(OR($H13="Code risk",$G13&gt;=5000),"High",IF(OR($H13="missing proof",$G13&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F13="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F13,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F13,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M13" s="2">
+        <f>IF(AND(AND(OR($F13="shortfall",$F13="damaged-goods",$F13="Shortfall / short-delivery",$F13="Damaged goods"),AND($C13&lt;&gt;"",$D13&lt;&gt;"",$D13-$C13&gt;30)),OR(UPPER($E13)="Y",UPPER($E13)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F13="shortfall",$F13="damaged-goods",$F13="Shortfall / short-delivery",$F13="Damaged goods"),AND($C13&lt;&gt;"",$D13&lt;&gt;"",$D13-$C13&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I13="missing proof","Await line-level proof from the retailer.",IF($I13="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I13="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N13">
+        <f>IF($F13="","",IF(AND(AND(OR($F13="shortfall",$F13="damaged-goods",$F13="Shortfall / short-delivery",$F13="Damaged goods"),AND($C13&lt;&gt;"",$D13&lt;&gt;"",$D13-$C13&gt;30)),OR(UPPER($E13)="Y",UPPER($E13)="YES")),"High",IF(OR($I13="Code risk",$H13&gt;=5000),"High",IF(OR($I13="missing proof",$H13&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1022,33 +1088,38 @@
           <t/>
         </is>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H14" s="3">
         <v>0</v>
       </c>
-      <c r="H14">
-        <f>IF($E14="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E14,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I14" s="2">
-        <f>IF($E14="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E14,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I14">
+        <f>IF($F14="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F14,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F14,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J14" s="2">
-        <f>IF($E14="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E14,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F14="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F14,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F14,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K14" s="2">
-        <f>IF($E14="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E14,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F14="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F14,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F14,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L14" s="2">
-        <f>IF(AND(OR($E14="shortfall",$E14="damaged-goods"),$C14&lt;&gt;"",$D14&lt;&gt;"",$D14-$C14&gt;30),"Claim raised more than 30 days after delivery.",IF($H14="missing proof","Await line-level proof from the retailer.",IF($H14="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H14="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M14">
-        <f>IF($E14="","",IF(AND(OR($E14="shortfall",$E14="damaged-goods"),$C14&lt;&gt;"",$D14&lt;&gt;"",$D14-$C14&gt;30),"High",IF(OR($H14="Code risk",$G14&gt;=5000),"High",IF(OR($H14="missing proof",$G14&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F14="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F14,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F14,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M14" s="2">
+        <f>IF(AND(AND(OR($F14="shortfall",$F14="damaged-goods",$F14="Shortfall / short-delivery",$F14="Damaged goods"),AND($C14&lt;&gt;"",$D14&lt;&gt;"",$D14-$C14&gt;30)),OR(UPPER($E14)="Y",UPPER($E14)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F14="shortfall",$F14="damaged-goods",$F14="Shortfall / short-delivery",$F14="Damaged goods"),AND($C14&lt;&gt;"",$D14&lt;&gt;"",$D14-$C14&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I14="missing proof","Await line-level proof from the retailer.",IF($I14="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I14="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N14">
+        <f>IF($F14="","",IF(AND(AND(OR($F14="shortfall",$F14="damaged-goods",$F14="Shortfall / short-delivery",$F14="Damaged goods"),AND($C14&lt;&gt;"",$D14&lt;&gt;"",$D14-$C14&gt;30)),OR(UPPER($E14)="Y",UPPER($E14)="YES")),"High",IF(OR($I14="Code risk",$H14&gt;=5000),"High",IF(OR($I14="missing proof",$H14&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1085,33 +1156,38 @@
           <t/>
         </is>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H15" s="3">
         <v>0</v>
       </c>
-      <c r="H15">
-        <f>IF($E15="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E15,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I15" s="2">
-        <f>IF($E15="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E15,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I15">
+        <f>IF($F15="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F15,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F15,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J15" s="2">
-        <f>IF($E15="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E15,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F15="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F15,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F15,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K15" s="2">
-        <f>IF($E15="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E15,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F15="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F15,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F15,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L15" s="2">
-        <f>IF(AND(OR($E15="shortfall",$E15="damaged-goods"),$C15&lt;&gt;"",$D15&lt;&gt;"",$D15-$C15&gt;30),"Claim raised more than 30 days after delivery.",IF($H15="missing proof","Await line-level proof from the retailer.",IF($H15="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H15="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M15">
-        <f>IF($E15="","",IF(AND(OR($E15="shortfall",$E15="damaged-goods"),$C15&lt;&gt;"",$D15&lt;&gt;"",$D15-$C15&gt;30),"High",IF(OR($H15="Code risk",$G15&gt;=5000),"High",IF(OR($H15="missing proof",$G15&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F15="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F15,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F15,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M15" s="2">
+        <f>IF(AND(AND(OR($F15="shortfall",$F15="damaged-goods",$F15="Shortfall / short-delivery",$F15="Damaged goods"),AND($C15&lt;&gt;"",$D15&lt;&gt;"",$D15-$C15&gt;30)),OR(UPPER($E15)="Y",UPPER($E15)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F15="shortfall",$F15="damaged-goods",$F15="Shortfall / short-delivery",$F15="Damaged goods"),AND($C15&lt;&gt;"",$D15&lt;&gt;"",$D15-$C15&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I15="missing proof","Await line-level proof from the retailer.",IF($I15="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I15="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N15">
+        <f>IF($F15="","",IF(AND(AND(OR($F15="shortfall",$F15="damaged-goods",$F15="Shortfall / short-delivery",$F15="Damaged goods"),AND($C15&lt;&gt;"",$D15&lt;&gt;"",$D15-$C15&gt;30)),OR(UPPER($E15)="Y",UPPER($E15)="YES")),"High",IF(OR($I15="Code risk",$H15&gt;=5000),"High",IF(OR($I15="missing proof",$H15&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1148,33 +1224,38 @@
           <t/>
         </is>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H16" s="3">
         <v>0</v>
       </c>
-      <c r="H16">
-        <f>IF($E16="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E16,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I16" s="2">
-        <f>IF($E16="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E16,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I16">
+        <f>IF($F16="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F16,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F16,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J16" s="2">
-        <f>IF($E16="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E16,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F16="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F16,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F16,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K16" s="2">
-        <f>IF($E16="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E16,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F16="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F16,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F16,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L16" s="2">
-        <f>IF(AND(OR($E16="shortfall",$E16="damaged-goods"),$C16&lt;&gt;"",$D16&lt;&gt;"",$D16-$C16&gt;30),"Claim raised more than 30 days after delivery.",IF($H16="missing proof","Await line-level proof from the retailer.",IF($H16="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H16="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M16">
-        <f>IF($E16="","",IF(AND(OR($E16="shortfall",$E16="damaged-goods"),$C16&lt;&gt;"",$D16&lt;&gt;"",$D16-$C16&gt;30),"High",IF(OR($H16="Code risk",$G16&gt;=5000),"High",IF(OR($H16="missing proof",$G16&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F16="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F16,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F16,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M16" s="2">
+        <f>IF(AND(AND(OR($F16="shortfall",$F16="damaged-goods",$F16="Shortfall / short-delivery",$F16="Damaged goods"),AND($C16&lt;&gt;"",$D16&lt;&gt;"",$D16-$C16&gt;30)),OR(UPPER($E16)="Y",UPPER($E16)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F16="shortfall",$F16="damaged-goods",$F16="Shortfall / short-delivery",$F16="Damaged goods"),AND($C16&lt;&gt;"",$D16&lt;&gt;"",$D16-$C16&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I16="missing proof","Await line-level proof from the retailer.",IF($I16="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I16="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N16">
+        <f>IF($F16="","",IF(AND(AND(OR($F16="shortfall",$F16="damaged-goods",$F16="Shortfall / short-delivery",$F16="Damaged goods"),AND($C16&lt;&gt;"",$D16&lt;&gt;"",$D16-$C16&gt;30)),OR(UPPER($E16)="Y",UPPER($E16)="YES")),"High",IF(OR($I16="Code risk",$H16&gt;=5000),"High",IF(OR($I16="missing proof",$H16&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1211,33 +1292,38 @@
           <t/>
         </is>
       </c>
-      <c r="G17" s="3">
+      <c r="G17" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H17" s="3">
         <v>0</v>
       </c>
-      <c r="H17">
-        <f>IF($E17="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E17,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I17" s="2">
-        <f>IF($E17="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E17,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I17">
+        <f>IF($F17="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F17,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F17,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J17" s="2">
-        <f>IF($E17="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E17,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F17="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F17,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F17,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K17" s="2">
-        <f>IF($E17="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E17,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F17="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F17,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F17,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L17" s="2">
-        <f>IF(AND(OR($E17="shortfall",$E17="damaged-goods"),$C17&lt;&gt;"",$D17&lt;&gt;"",$D17-$C17&gt;30),"Claim raised more than 30 days after delivery.",IF($H17="missing proof","Await line-level proof from the retailer.",IF($H17="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H17="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M17">
-        <f>IF($E17="","",IF(AND(OR($E17="shortfall",$E17="damaged-goods"),$C17&lt;&gt;"",$D17&lt;&gt;"",$D17-$C17&gt;30),"High",IF(OR($H17="Code risk",$G17&gt;=5000),"High",IF(OR($H17="missing proof",$G17&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F17="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F17,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F17,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M17" s="2">
+        <f>IF(AND(AND(OR($F17="shortfall",$F17="damaged-goods",$F17="Shortfall / short-delivery",$F17="Damaged goods"),AND($C17&lt;&gt;"",$D17&lt;&gt;"",$D17-$C17&gt;30)),OR(UPPER($E17)="Y",UPPER($E17)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F17="shortfall",$F17="damaged-goods",$F17="Shortfall / short-delivery",$F17="Damaged goods"),AND($C17&lt;&gt;"",$D17&lt;&gt;"",$D17-$C17&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I17="missing proof","Await line-level proof from the retailer.",IF($I17="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I17="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N17">
+        <f>IF($F17="","",IF(AND(AND(OR($F17="shortfall",$F17="damaged-goods",$F17="Shortfall / short-delivery",$F17="Damaged goods"),AND($C17&lt;&gt;"",$D17&lt;&gt;"",$D17-$C17&gt;30)),OR(UPPER($E17)="Y",UPPER($E17)="YES")),"High",IF(OR($I17="Code risk",$H17&gt;=5000),"High",IF(OR($I17="missing proof",$H17&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1274,33 +1360,38 @@
           <t/>
         </is>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H18" s="3">
         <v>0</v>
       </c>
-      <c r="H18">
-        <f>IF($E18="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E18,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I18" s="2">
-        <f>IF($E18="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E18,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I18">
+        <f>IF($F18="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F18,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F18,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J18" s="2">
-        <f>IF($E18="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E18,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F18="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F18,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F18,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K18" s="2">
-        <f>IF($E18="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E18,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F18="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F18,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F18,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L18" s="2">
-        <f>IF(AND(OR($E18="shortfall",$E18="damaged-goods"),$C18&lt;&gt;"",$D18&lt;&gt;"",$D18-$C18&gt;30),"Claim raised more than 30 days after delivery.",IF($H18="missing proof","Await line-level proof from the retailer.",IF($H18="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H18="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M18">
-        <f>IF($E18="","",IF(AND(OR($E18="shortfall",$E18="damaged-goods"),$C18&lt;&gt;"",$D18&lt;&gt;"",$D18-$C18&gt;30),"High",IF(OR($H18="Code risk",$G18&gt;=5000),"High",IF(OR($H18="missing proof",$G18&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F18="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F18,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F18,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M18" s="2">
+        <f>IF(AND(AND(OR($F18="shortfall",$F18="damaged-goods",$F18="Shortfall / short-delivery",$F18="Damaged goods"),AND($C18&lt;&gt;"",$D18&lt;&gt;"",$D18-$C18&gt;30)),OR(UPPER($E18)="Y",UPPER($E18)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F18="shortfall",$F18="damaged-goods",$F18="Shortfall / short-delivery",$F18="Damaged goods"),AND($C18&lt;&gt;"",$D18&lt;&gt;"",$D18-$C18&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I18="missing proof","Await line-level proof from the retailer.",IF($I18="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I18="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N18">
+        <f>IF($F18="","",IF(AND(AND(OR($F18="shortfall",$F18="damaged-goods",$F18="Shortfall / short-delivery",$F18="Damaged goods"),AND($C18&lt;&gt;"",$D18&lt;&gt;"",$D18-$C18&gt;30)),OR(UPPER($E18)="Y",UPPER($E18)="YES")),"High",IF(OR($I18="Code risk",$H18&gt;=5000),"High",IF(OR($I18="missing proof",$H18&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1337,33 +1428,38 @@
           <t/>
         </is>
       </c>
-      <c r="G19" s="3">
+      <c r="G19" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H19" s="3">
         <v>0</v>
       </c>
-      <c r="H19">
-        <f>IF($E19="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E19,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I19" s="2">
-        <f>IF($E19="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E19,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I19">
+        <f>IF($F19="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F19,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F19,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J19" s="2">
-        <f>IF($E19="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E19,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F19="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F19,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F19,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K19" s="2">
-        <f>IF($E19="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E19,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F19="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F19,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F19,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L19" s="2">
-        <f>IF(AND(OR($E19="shortfall",$E19="damaged-goods"),$C19&lt;&gt;"",$D19&lt;&gt;"",$D19-$C19&gt;30),"Claim raised more than 30 days after delivery.",IF($H19="missing proof","Await line-level proof from the retailer.",IF($H19="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H19="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M19">
-        <f>IF($E19="","",IF(AND(OR($E19="shortfall",$E19="damaged-goods"),$C19&lt;&gt;"",$D19&lt;&gt;"",$D19-$C19&gt;30),"High",IF(OR($H19="Code risk",$G19&gt;=5000),"High",IF(OR($H19="missing proof",$G19&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F19="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F19,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F19,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M19" s="2">
+        <f>IF(AND(AND(OR($F19="shortfall",$F19="damaged-goods",$F19="Shortfall / short-delivery",$F19="Damaged goods"),AND($C19&lt;&gt;"",$D19&lt;&gt;"",$D19-$C19&gt;30)),OR(UPPER($E19)="Y",UPPER($E19)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F19="shortfall",$F19="damaged-goods",$F19="Shortfall / short-delivery",$F19="Damaged goods"),AND($C19&lt;&gt;"",$D19&lt;&gt;"",$D19-$C19&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I19="missing proof","Await line-level proof from the retailer.",IF($I19="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I19="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N19">
+        <f>IF($F19="","",IF(AND(AND(OR($F19="shortfall",$F19="damaged-goods",$F19="Shortfall / short-delivery",$F19="Damaged goods"),AND($C19&lt;&gt;"",$D19&lt;&gt;"",$D19-$C19&gt;30)),OR(UPPER($E19)="Y",UPPER($E19)="YES")),"High",IF(OR($I19="Code risk",$H19&gt;=5000),"High",IF(OR($I19="missing proof",$H19&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1400,33 +1496,38 @@
           <t/>
         </is>
       </c>
-      <c r="G20" s="3">
+      <c r="G20" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H20" s="3">
         <v>0</v>
       </c>
-      <c r="H20">
-        <f>IF($E20="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E20,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I20" s="2">
-        <f>IF($E20="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E20,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I20">
+        <f>IF($F20="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F20,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F20,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J20" s="2">
-        <f>IF($E20="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E20,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F20="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F20,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F20,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K20" s="2">
-        <f>IF($E20="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E20,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F20="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F20,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F20,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L20" s="2">
-        <f>IF(AND(OR($E20="shortfall",$E20="damaged-goods"),$C20&lt;&gt;"",$D20&lt;&gt;"",$D20-$C20&gt;30),"Claim raised more than 30 days after delivery.",IF($H20="missing proof","Await line-level proof from the retailer.",IF($H20="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H20="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M20">
-        <f>IF($E20="","",IF(AND(OR($E20="shortfall",$E20="damaged-goods"),$C20&lt;&gt;"",$D20&lt;&gt;"",$D20-$C20&gt;30),"High",IF(OR($H20="Code risk",$G20&gt;=5000),"High",IF(OR($H20="missing proof",$G20&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F20="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F20,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F20,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M20" s="2">
+        <f>IF(AND(AND(OR($F20="shortfall",$F20="damaged-goods",$F20="Shortfall / short-delivery",$F20="Damaged goods"),AND($C20&lt;&gt;"",$D20&lt;&gt;"",$D20-$C20&gt;30)),OR(UPPER($E20)="Y",UPPER($E20)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F20="shortfall",$F20="damaged-goods",$F20="Shortfall / short-delivery",$F20="Damaged goods"),AND($C20&lt;&gt;"",$D20&lt;&gt;"",$D20-$C20&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I20="missing proof","Await line-level proof from the retailer.",IF($I20="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I20="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N20">
+        <f>IF($F20="","",IF(AND(AND(OR($F20="shortfall",$F20="damaged-goods",$F20="Shortfall / short-delivery",$F20="Damaged goods"),AND($C20&lt;&gt;"",$D20&lt;&gt;"",$D20-$C20&gt;30)),OR(UPPER($E20)="Y",UPPER($E20)="YES")),"High",IF(OR($I20="Code risk",$H20&gt;=5000),"High",IF(OR($I20="missing proof",$H20&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1463,33 +1564,38 @@
           <t/>
         </is>
       </c>
-      <c r="G21" s="3">
+      <c r="G21" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H21" s="3">
         <v>0</v>
       </c>
-      <c r="H21">
-        <f>IF($E21="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E21,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I21" s="2">
-        <f>IF($E21="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E21,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I21">
+        <f>IF($F21="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F21,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F21,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J21" s="2">
-        <f>IF($E21="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E21,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F21="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F21,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F21,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K21" s="2">
-        <f>IF($E21="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E21,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F21="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F21,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F21,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L21" s="2">
-        <f>IF(AND(OR($E21="shortfall",$E21="damaged-goods"),$C21&lt;&gt;"",$D21&lt;&gt;"",$D21-$C21&gt;30),"Claim raised more than 30 days after delivery.",IF($H21="missing proof","Await line-level proof from the retailer.",IF($H21="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H21="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M21">
-        <f>IF($E21="","",IF(AND(OR($E21="shortfall",$E21="damaged-goods"),$C21&lt;&gt;"",$D21&lt;&gt;"",$D21-$C21&gt;30),"High",IF(OR($H21="Code risk",$G21&gt;=5000),"High",IF(OR($H21="missing proof",$G21&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F21="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F21,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F21,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M21" s="2">
+        <f>IF(AND(AND(OR($F21="shortfall",$F21="damaged-goods",$F21="Shortfall / short-delivery",$F21="Damaged goods"),AND($C21&lt;&gt;"",$D21&lt;&gt;"",$D21-$C21&gt;30)),OR(UPPER($E21)="Y",UPPER($E21)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F21="shortfall",$F21="damaged-goods",$F21="Shortfall / short-delivery",$F21="Damaged goods"),AND($C21&lt;&gt;"",$D21&lt;&gt;"",$D21-$C21&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I21="missing proof","Await line-level proof from the retailer.",IF($I21="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I21="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N21">
+        <f>IF($F21="","",IF(AND(AND(OR($F21="shortfall",$F21="damaged-goods",$F21="Shortfall / short-delivery",$F21="Damaged goods"),AND($C21&lt;&gt;"",$D21&lt;&gt;"",$D21-$C21&gt;30)),OR(UPPER($E21)="Y",UPPER($E21)="YES")),"High",IF(OR($I21="Code risk",$H21&gt;=5000),"High",IF(OR($I21="missing proof",$H21&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1526,33 +1632,38 @@
           <t/>
         </is>
       </c>
-      <c r="G22" s="3">
+      <c r="G22" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H22" s="3">
         <v>0</v>
       </c>
-      <c r="H22">
-        <f>IF($E22="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E22,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I22" s="2">
-        <f>IF($E22="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E22,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I22">
+        <f>IF($F22="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F22,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F22,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J22" s="2">
-        <f>IF($E22="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E22,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F22="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F22,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F22,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K22" s="2">
-        <f>IF($E22="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E22,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F22="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F22,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F22,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L22" s="2">
-        <f>IF(AND(OR($E22="shortfall",$E22="damaged-goods"),$C22&lt;&gt;"",$D22&lt;&gt;"",$D22-$C22&gt;30),"Claim raised more than 30 days after delivery.",IF($H22="missing proof","Await line-level proof from the retailer.",IF($H22="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H22="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M22">
-        <f>IF($E22="","",IF(AND(OR($E22="shortfall",$E22="damaged-goods"),$C22&lt;&gt;"",$D22&lt;&gt;"",$D22-$C22&gt;30),"High",IF(OR($H22="Code risk",$G22&gt;=5000),"High",IF(OR($H22="missing proof",$G22&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F22="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F22,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F22,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M22" s="2">
+        <f>IF(AND(AND(OR($F22="shortfall",$F22="damaged-goods",$F22="Shortfall / short-delivery",$F22="Damaged goods"),AND($C22&lt;&gt;"",$D22&lt;&gt;"",$D22-$C22&gt;30)),OR(UPPER($E22)="Y",UPPER($E22)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F22="shortfall",$F22="damaged-goods",$F22="Shortfall / short-delivery",$F22="Damaged goods"),AND($C22&lt;&gt;"",$D22&lt;&gt;"",$D22-$C22&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I22="missing proof","Await line-level proof from the retailer.",IF($I22="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I22="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N22">
+        <f>IF($F22="","",IF(AND(AND(OR($F22="shortfall",$F22="damaged-goods",$F22="Shortfall / short-delivery",$F22="Damaged goods"),AND($C22&lt;&gt;"",$D22&lt;&gt;"",$D22-$C22&gt;30)),OR(UPPER($E22)="Y",UPPER($E22)="YES")),"High",IF(OR($I22="Code risk",$H22&gt;=5000),"High",IF(OR($I22="missing proof",$H22&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1589,33 +1700,38 @@
           <t/>
         </is>
       </c>
-      <c r="G23" s="3">
+      <c r="G23" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H23" s="3">
         <v>0</v>
       </c>
-      <c r="H23">
-        <f>IF($E23="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E23,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I23" s="2">
-        <f>IF($E23="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E23,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I23">
+        <f>IF($F23="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F23,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F23,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J23" s="2">
-        <f>IF($E23="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E23,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F23="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F23,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F23,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K23" s="2">
-        <f>IF($E23="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E23,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F23="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F23,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F23,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L23" s="2">
-        <f>IF(AND(OR($E23="shortfall",$E23="damaged-goods"),$C23&lt;&gt;"",$D23&lt;&gt;"",$D23-$C23&gt;30),"Claim raised more than 30 days after delivery.",IF($H23="missing proof","Await line-level proof from the retailer.",IF($H23="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H23="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M23">
-        <f>IF($E23="","",IF(AND(OR($E23="shortfall",$E23="damaged-goods"),$C23&lt;&gt;"",$D23&lt;&gt;"",$D23-$C23&gt;30),"High",IF(OR($H23="Code risk",$G23&gt;=5000),"High",IF(OR($H23="missing proof",$G23&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F23="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F23,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F23,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M23" s="2">
+        <f>IF(AND(AND(OR($F23="shortfall",$F23="damaged-goods",$F23="Shortfall / short-delivery",$F23="Damaged goods"),AND($C23&lt;&gt;"",$D23&lt;&gt;"",$D23-$C23&gt;30)),OR(UPPER($E23)="Y",UPPER($E23)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F23="shortfall",$F23="damaged-goods",$F23="Shortfall / short-delivery",$F23="Damaged goods"),AND($C23&lt;&gt;"",$D23&lt;&gt;"",$D23-$C23&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I23="missing proof","Await line-level proof from the retailer.",IF($I23="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I23="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N23">
+        <f>IF($F23="","",IF(AND(AND(OR($F23="shortfall",$F23="damaged-goods",$F23="Shortfall / short-delivery",$F23="Damaged goods"),AND($C23&lt;&gt;"",$D23&lt;&gt;"",$D23-$C23&gt;30)),OR(UPPER($E23)="Y",UPPER($E23)="YES")),"High",IF(OR($I23="Code risk",$H23&gt;=5000),"High",IF(OR($I23="missing proof",$H23&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1652,33 +1768,38 @@
           <t/>
         </is>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H24" s="3">
         <v>0</v>
       </c>
-      <c r="H24">
-        <f>IF($E24="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E24,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I24" s="2">
-        <f>IF($E24="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E24,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I24">
+        <f>IF($F24="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F24,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F24,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J24" s="2">
-        <f>IF($E24="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E24,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F24="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F24,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F24,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K24" s="2">
-        <f>IF($E24="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E24,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F24="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F24,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F24,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L24" s="2">
-        <f>IF(AND(OR($E24="shortfall",$E24="damaged-goods"),$C24&lt;&gt;"",$D24&lt;&gt;"",$D24-$C24&gt;30),"Claim raised more than 30 days after delivery.",IF($H24="missing proof","Await line-level proof from the retailer.",IF($H24="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H24="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M24">
-        <f>IF($E24="","",IF(AND(OR($E24="shortfall",$E24="damaged-goods"),$C24&lt;&gt;"",$D24&lt;&gt;"",$D24-$C24&gt;30),"High",IF(OR($H24="Code risk",$G24&gt;=5000),"High",IF(OR($H24="missing proof",$G24&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F24="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F24,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F24,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M24" s="2">
+        <f>IF(AND(AND(OR($F24="shortfall",$F24="damaged-goods",$F24="Shortfall / short-delivery",$F24="Damaged goods"),AND($C24&lt;&gt;"",$D24&lt;&gt;"",$D24-$C24&gt;30)),OR(UPPER($E24)="Y",UPPER($E24)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F24="shortfall",$F24="damaged-goods",$F24="Shortfall / short-delivery",$F24="Damaged goods"),AND($C24&lt;&gt;"",$D24&lt;&gt;"",$D24-$C24&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I24="missing proof","Await line-level proof from the retailer.",IF($I24="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I24="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N24">
+        <f>IF($F24="","",IF(AND(AND(OR($F24="shortfall",$F24="damaged-goods",$F24="Shortfall / short-delivery",$F24="Damaged goods"),AND($C24&lt;&gt;"",$D24&lt;&gt;"",$D24-$C24&gt;30)),OR(UPPER($E24)="Y",UPPER($E24)="YES")),"High",IF(OR($I24="Code risk",$H24&gt;=5000),"High",IF(OR($I24="missing proof",$H24&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1715,33 +1836,38 @@
           <t/>
         </is>
       </c>
-      <c r="G25" s="3">
+      <c r="G25" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H25" s="3">
         <v>0</v>
       </c>
-      <c r="H25">
-        <f>IF($E25="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E25,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I25" s="2">
-        <f>IF($E25="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E25,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I25">
+        <f>IF($F25="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F25,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F25,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J25" s="2">
-        <f>IF($E25="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E25,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F25="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F25,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F25,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K25" s="2">
-        <f>IF($E25="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E25,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F25="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F25,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F25,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L25" s="2">
-        <f>IF(AND(OR($E25="shortfall",$E25="damaged-goods"),$C25&lt;&gt;"",$D25&lt;&gt;"",$D25-$C25&gt;30),"Claim raised more than 30 days after delivery.",IF($H25="missing proof","Await line-level proof from the retailer.",IF($H25="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H25="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M25">
-        <f>IF($E25="","",IF(AND(OR($E25="shortfall",$E25="damaged-goods"),$C25&lt;&gt;"",$D25&lt;&gt;"",$D25-$C25&gt;30),"High",IF(OR($H25="Code risk",$G25&gt;=5000),"High",IF(OR($H25="missing proof",$G25&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F25="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F25,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F25,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M25" s="2">
+        <f>IF(AND(AND(OR($F25="shortfall",$F25="damaged-goods",$F25="Shortfall / short-delivery",$F25="Damaged goods"),AND($C25&lt;&gt;"",$D25&lt;&gt;"",$D25-$C25&gt;30)),OR(UPPER($E25)="Y",UPPER($E25)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F25="shortfall",$F25="damaged-goods",$F25="Shortfall / short-delivery",$F25="Damaged goods"),AND($C25&lt;&gt;"",$D25&lt;&gt;"",$D25-$C25&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I25="missing proof","Await line-level proof from the retailer.",IF($I25="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I25="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N25">
+        <f>IF($F25="","",IF(AND(AND(OR($F25="shortfall",$F25="damaged-goods",$F25="Shortfall / short-delivery",$F25="Damaged goods"),AND($C25&lt;&gt;"",$D25&lt;&gt;"",$D25-$C25&gt;30)),OR(UPPER($E25)="Y",UPPER($E25)="YES")),"High",IF(OR($I25="Code risk",$H25&gt;=5000),"High",IF(OR($I25="missing proof",$H25&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1778,33 +1904,38 @@
           <t/>
         </is>
       </c>
-      <c r="G26" s="3">
+      <c r="G26" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H26" s="3">
         <v>0</v>
       </c>
-      <c r="H26">
-        <f>IF($E26="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E26,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I26" s="2">
-        <f>IF($E26="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E26,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I26">
+        <f>IF($F26="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F26,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F26,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J26" s="2">
-        <f>IF($E26="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E26,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F26="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F26,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F26,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K26" s="2">
-        <f>IF($E26="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E26,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F26="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F26,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F26,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L26" s="2">
-        <f>IF(AND(OR($E26="shortfall",$E26="damaged-goods"),$C26&lt;&gt;"",$D26&lt;&gt;"",$D26-$C26&gt;30),"Claim raised more than 30 days after delivery.",IF($H26="missing proof","Await line-level proof from the retailer.",IF($H26="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H26="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M26">
-        <f>IF($E26="","",IF(AND(OR($E26="shortfall",$E26="damaged-goods"),$C26&lt;&gt;"",$D26&lt;&gt;"",$D26-$C26&gt;30),"High",IF(OR($H26="Code risk",$G26&gt;=5000),"High",IF(OR($H26="missing proof",$G26&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F26="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F26,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F26,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M26" s="2">
+        <f>IF(AND(AND(OR($F26="shortfall",$F26="damaged-goods",$F26="Shortfall / short-delivery",$F26="Damaged goods"),AND($C26&lt;&gt;"",$D26&lt;&gt;"",$D26-$C26&gt;30)),OR(UPPER($E26)="Y",UPPER($E26)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F26="shortfall",$F26="damaged-goods",$F26="Shortfall / short-delivery",$F26="Damaged goods"),AND($C26&lt;&gt;"",$D26&lt;&gt;"",$D26-$C26&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I26="missing proof","Await line-level proof from the retailer.",IF($I26="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I26="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N26">
+        <f>IF($F26="","",IF(AND(AND(OR($F26="shortfall",$F26="damaged-goods",$F26="Shortfall / short-delivery",$F26="Damaged goods"),AND($C26&lt;&gt;"",$D26&lt;&gt;"",$D26-$C26&gt;30)),OR(UPPER($E26)="Y",UPPER($E26)="YES")),"High",IF(OR($I26="Code risk",$H26&gt;=5000),"High",IF(OR($I26="missing proof",$H26&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1841,33 +1972,38 @@
           <t/>
         </is>
       </c>
-      <c r="G27" s="3">
+      <c r="G27" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H27" s="3">
         <v>0</v>
       </c>
-      <c r="H27">
-        <f>IF($E27="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E27,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I27" s="2">
-        <f>IF($E27="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E27,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I27">
+        <f>IF($F27="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F27,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F27,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J27" s="2">
-        <f>IF($E27="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E27,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F27="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F27,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F27,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K27" s="2">
-        <f>IF($E27="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E27,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F27="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F27,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F27,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L27" s="2">
-        <f>IF(AND(OR($E27="shortfall",$E27="damaged-goods"),$C27&lt;&gt;"",$D27&lt;&gt;"",$D27-$C27&gt;30),"Claim raised more than 30 days after delivery.",IF($H27="missing proof","Await line-level proof from the retailer.",IF($H27="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H27="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M27">
-        <f>IF($E27="","",IF(AND(OR($E27="shortfall",$E27="damaged-goods"),$C27&lt;&gt;"",$D27&lt;&gt;"",$D27-$C27&gt;30),"High",IF(OR($H27="Code risk",$G27&gt;=5000),"High",IF(OR($H27="missing proof",$G27&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F27="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F27,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F27,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M27" s="2">
+        <f>IF(AND(AND(OR($F27="shortfall",$F27="damaged-goods",$F27="Shortfall / short-delivery",$F27="Damaged goods"),AND($C27&lt;&gt;"",$D27&lt;&gt;"",$D27-$C27&gt;30)),OR(UPPER($E27)="Y",UPPER($E27)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F27="shortfall",$F27="damaged-goods",$F27="Shortfall / short-delivery",$F27="Damaged goods"),AND($C27&lt;&gt;"",$D27&lt;&gt;"",$D27-$C27&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I27="missing proof","Await line-level proof from the retailer.",IF($I27="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I27="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N27">
+        <f>IF($F27="","",IF(AND(AND(OR($F27="shortfall",$F27="damaged-goods",$F27="Shortfall / short-delivery",$F27="Damaged goods"),AND($C27&lt;&gt;"",$D27&lt;&gt;"",$D27-$C27&gt;30)),OR(UPPER($E27)="Y",UPPER($E27)="YES")),"High",IF(OR($I27="Code risk",$H27&gt;=5000),"High",IF(OR($I27="missing proof",$H27&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1904,33 +2040,38 @@
           <t/>
         </is>
       </c>
-      <c r="G28" s="3">
+      <c r="G28" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H28" s="3">
         <v>0</v>
       </c>
-      <c r="H28">
-        <f>IF($E28="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E28,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I28" s="2">
-        <f>IF($E28="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E28,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I28">
+        <f>IF($F28="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F28,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F28,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J28" s="2">
-        <f>IF($E28="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E28,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F28="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F28,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F28,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K28" s="2">
-        <f>IF($E28="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E28,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F28="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F28,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F28,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L28" s="2">
-        <f>IF(AND(OR($E28="shortfall",$E28="damaged-goods"),$C28&lt;&gt;"",$D28&lt;&gt;"",$D28-$C28&gt;30),"Claim raised more than 30 days after delivery.",IF($H28="missing proof","Await line-level proof from the retailer.",IF($H28="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H28="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M28">
-        <f>IF($E28="","",IF(AND(OR($E28="shortfall",$E28="damaged-goods"),$C28&lt;&gt;"",$D28&lt;&gt;"",$D28-$C28&gt;30),"High",IF(OR($H28="Code risk",$G28&gt;=5000),"High",IF(OR($H28="missing proof",$G28&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F28="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F28,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F28,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M28" s="2">
+        <f>IF(AND(AND(OR($F28="shortfall",$F28="damaged-goods",$F28="Shortfall / short-delivery",$F28="Damaged goods"),AND($C28&lt;&gt;"",$D28&lt;&gt;"",$D28-$C28&gt;30)),OR(UPPER($E28)="Y",UPPER($E28)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F28="shortfall",$F28="damaged-goods",$F28="Shortfall / short-delivery",$F28="Damaged goods"),AND($C28&lt;&gt;"",$D28&lt;&gt;"",$D28-$C28&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I28="missing proof","Await line-level proof from the retailer.",IF($I28="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I28="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N28">
+        <f>IF($F28="","",IF(AND(AND(OR($F28="shortfall",$F28="damaged-goods",$F28="Shortfall / short-delivery",$F28="Damaged goods"),AND($C28&lt;&gt;"",$D28&lt;&gt;"",$D28-$C28&gt;30)),OR(UPPER($E28)="Y",UPPER($E28)="YES")),"High",IF(OR($I28="Code risk",$H28&gt;=5000),"High",IF(OR($I28="missing proof",$H28&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1967,33 +2108,38 @@
           <t/>
         </is>
       </c>
-      <c r="G29" s="3">
+      <c r="G29" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H29" s="3">
         <v>0</v>
       </c>
-      <c r="H29">
-        <f>IF($E29="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E29,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I29" s="2">
-        <f>IF($E29="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E29,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I29">
+        <f>IF($F29="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F29,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F29,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J29" s="2">
-        <f>IF($E29="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E29,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F29="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F29,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F29,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K29" s="2">
-        <f>IF($E29="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E29,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F29="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F29,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F29,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L29" s="2">
-        <f>IF(AND(OR($E29="shortfall",$E29="damaged-goods"),$C29&lt;&gt;"",$D29&lt;&gt;"",$D29-$C29&gt;30),"Claim raised more than 30 days after delivery.",IF($H29="missing proof","Await line-level proof from the retailer.",IF($H29="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H29="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M29">
-        <f>IF($E29="","",IF(AND(OR($E29="shortfall",$E29="damaged-goods"),$C29&lt;&gt;"",$D29&lt;&gt;"",$D29-$C29&gt;30),"High",IF(OR($H29="Code risk",$G29&gt;=5000),"High",IF(OR($H29="missing proof",$G29&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F29="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F29,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F29,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M29" s="2">
+        <f>IF(AND(AND(OR($F29="shortfall",$F29="damaged-goods",$F29="Shortfall / short-delivery",$F29="Damaged goods"),AND($C29&lt;&gt;"",$D29&lt;&gt;"",$D29-$C29&gt;30)),OR(UPPER($E29)="Y",UPPER($E29)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F29="shortfall",$F29="damaged-goods",$F29="Shortfall / short-delivery",$F29="Damaged goods"),AND($C29&lt;&gt;"",$D29&lt;&gt;"",$D29-$C29&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I29="missing proof","Await line-level proof from the retailer.",IF($I29="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I29="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N29">
+        <f>IF($F29="","",IF(AND(AND(OR($F29="shortfall",$F29="damaged-goods",$F29="Shortfall / short-delivery",$F29="Damaged goods"),AND($C29&lt;&gt;"",$D29&lt;&gt;"",$D29-$C29&gt;30)),OR(UPPER($E29)="Y",UPPER($E29)="YES")),"High",IF(OR($I29="Code risk",$H29&gt;=5000),"High",IF(OR($I29="missing proof",$H29&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2030,33 +2176,38 @@
           <t/>
         </is>
       </c>
-      <c r="G30" s="3">
+      <c r="G30" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H30" s="3">
         <v>0</v>
       </c>
-      <c r="H30">
-        <f>IF($E30="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E30,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I30" s="2">
-        <f>IF($E30="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E30,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I30">
+        <f>IF($F30="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F30,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F30,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J30" s="2">
-        <f>IF($E30="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E30,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F30="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F30,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F30,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K30" s="2">
-        <f>IF($E30="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E30,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F30="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F30,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F30,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L30" s="2">
-        <f>IF(AND(OR($E30="shortfall",$E30="damaged-goods"),$C30&lt;&gt;"",$D30&lt;&gt;"",$D30-$C30&gt;30),"Claim raised more than 30 days after delivery.",IF($H30="missing proof","Await line-level proof from the retailer.",IF($H30="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H30="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M30">
-        <f>IF($E30="","",IF(AND(OR($E30="shortfall",$E30="damaged-goods"),$C30&lt;&gt;"",$D30&lt;&gt;"",$D30-$C30&gt;30),"High",IF(OR($H30="Code risk",$G30&gt;=5000),"High",IF(OR($H30="missing proof",$G30&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F30="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F30,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F30,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M30" s="2">
+        <f>IF(AND(AND(OR($F30="shortfall",$F30="damaged-goods",$F30="Shortfall / short-delivery",$F30="Damaged goods"),AND($C30&lt;&gt;"",$D30&lt;&gt;"",$D30-$C30&gt;30)),OR(UPPER($E30)="Y",UPPER($E30)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F30="shortfall",$F30="damaged-goods",$F30="Shortfall / short-delivery",$F30="Damaged goods"),AND($C30&lt;&gt;"",$D30&lt;&gt;"",$D30-$C30&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I30="missing proof","Await line-level proof from the retailer.",IF($I30="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I30="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N30">
+        <f>IF($F30="","",IF(AND(AND(OR($F30="shortfall",$F30="damaged-goods",$F30="Shortfall / short-delivery",$F30="Damaged goods"),AND($C30&lt;&gt;"",$D30&lt;&gt;"",$D30-$C30&gt;30)),OR(UPPER($E30)="Y",UPPER($E30)="YES")),"High",IF(OR($I30="Code risk",$H30&gt;=5000),"High",IF(OR($I30="missing proof",$H30&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2093,33 +2244,38 @@
           <t/>
         </is>
       </c>
-      <c r="G31" s="3">
+      <c r="G31" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H31" s="3">
         <v>0</v>
       </c>
-      <c r="H31">
-        <f>IF($E31="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E31,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I31" s="2">
-        <f>IF($E31="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E31,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I31">
+        <f>IF($F31="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F31,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F31,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J31" s="2">
-        <f>IF($E31="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E31,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F31="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F31,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F31,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K31" s="2">
-        <f>IF($E31="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E31,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F31="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F31,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F31,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L31" s="2">
-        <f>IF(AND(OR($E31="shortfall",$E31="damaged-goods"),$C31&lt;&gt;"",$D31&lt;&gt;"",$D31-$C31&gt;30),"Claim raised more than 30 days after delivery.",IF($H31="missing proof","Await line-level proof from the retailer.",IF($H31="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H31="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M31">
-        <f>IF($E31="","",IF(AND(OR($E31="shortfall",$E31="damaged-goods"),$C31&lt;&gt;"",$D31&lt;&gt;"",$D31-$C31&gt;30),"High",IF(OR($H31="Code risk",$G31&gt;=5000),"High",IF(OR($H31="missing proof",$G31&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F31="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F31,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F31,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M31" s="2">
+        <f>IF(AND(AND(OR($F31="shortfall",$F31="damaged-goods",$F31="Shortfall / short-delivery",$F31="Damaged goods"),AND($C31&lt;&gt;"",$D31&lt;&gt;"",$D31-$C31&gt;30)),OR(UPPER($E31)="Y",UPPER($E31)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F31="shortfall",$F31="damaged-goods",$F31="Shortfall / short-delivery",$F31="Damaged goods"),AND($C31&lt;&gt;"",$D31&lt;&gt;"",$D31-$C31&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I31="missing proof","Await line-level proof from the retailer.",IF($I31="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I31="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N31">
+        <f>IF($F31="","",IF(AND(AND(OR($F31="shortfall",$F31="damaged-goods",$F31="Shortfall / short-delivery",$F31="Damaged goods"),AND($C31&lt;&gt;"",$D31&lt;&gt;"",$D31-$C31&gt;30)),OR(UPPER($E31)="Y",UPPER($E31)="YES")),"High",IF(OR($I31="Code risk",$H31&gt;=5000),"High",IF(OR($I31="missing proof",$H31&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2156,33 +2312,38 @@
           <t/>
         </is>
       </c>
-      <c r="G32" s="3">
+      <c r="G32" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H32" s="3">
         <v>0</v>
       </c>
-      <c r="H32">
-        <f>IF($E32="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E32,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I32" s="2">
-        <f>IF($E32="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E32,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I32">
+        <f>IF($F32="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F32,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F32,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J32" s="2">
-        <f>IF($E32="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E32,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F32="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F32,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F32,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K32" s="2">
-        <f>IF($E32="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E32,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F32="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F32,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F32,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L32" s="2">
-        <f>IF(AND(OR($E32="shortfall",$E32="damaged-goods"),$C32&lt;&gt;"",$D32&lt;&gt;"",$D32-$C32&gt;30),"Claim raised more than 30 days after delivery.",IF($H32="missing proof","Await line-level proof from the retailer.",IF($H32="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H32="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M32">
-        <f>IF($E32="","",IF(AND(OR($E32="shortfall",$E32="damaged-goods"),$C32&lt;&gt;"",$D32&lt;&gt;"",$D32-$C32&gt;30),"High",IF(OR($H32="Code risk",$G32&gt;=5000),"High",IF(OR($H32="missing proof",$G32&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F32="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F32,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F32,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M32" s="2">
+        <f>IF(AND(AND(OR($F32="shortfall",$F32="damaged-goods",$F32="Shortfall / short-delivery",$F32="Damaged goods"),AND($C32&lt;&gt;"",$D32&lt;&gt;"",$D32-$C32&gt;30)),OR(UPPER($E32)="Y",UPPER($E32)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F32="shortfall",$F32="damaged-goods",$F32="Shortfall / short-delivery",$F32="Damaged goods"),AND($C32&lt;&gt;"",$D32&lt;&gt;"",$D32-$C32&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I32="missing proof","Await line-level proof from the retailer.",IF($I32="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I32="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N32">
+        <f>IF($F32="","",IF(AND(AND(OR($F32="shortfall",$F32="damaged-goods",$F32="Shortfall / short-delivery",$F32="Damaged goods"),AND($C32&lt;&gt;"",$D32&lt;&gt;"",$D32-$C32&gt;30)),OR(UPPER($E32)="Y",UPPER($E32)="YES")),"High",IF(OR($I32="Code risk",$H32&gt;=5000),"High",IF(OR($I32="missing proof",$H32&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2219,33 +2380,38 @@
           <t/>
         </is>
       </c>
-      <c r="G33" s="3">
+      <c r="G33" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H33" s="3">
         <v>0</v>
       </c>
-      <c r="H33">
-        <f>IF($E33="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E33,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I33" s="2">
-        <f>IF($E33="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E33,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I33">
+        <f>IF($F33="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F33,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F33,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J33" s="2">
-        <f>IF($E33="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E33,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F33="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F33,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F33,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K33" s="2">
-        <f>IF($E33="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E33,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F33="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F33,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F33,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L33" s="2">
-        <f>IF(AND(OR($E33="shortfall",$E33="damaged-goods"),$C33&lt;&gt;"",$D33&lt;&gt;"",$D33-$C33&gt;30),"Claim raised more than 30 days after delivery.",IF($H33="missing proof","Await line-level proof from the retailer.",IF($H33="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H33="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M33">
-        <f>IF($E33="","",IF(AND(OR($E33="shortfall",$E33="damaged-goods"),$C33&lt;&gt;"",$D33&lt;&gt;"",$D33-$C33&gt;30),"High",IF(OR($H33="Code risk",$G33&gt;=5000),"High",IF(OR($H33="missing proof",$G33&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F33="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F33,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F33,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M33" s="2">
+        <f>IF(AND(AND(OR($F33="shortfall",$F33="damaged-goods",$F33="Shortfall / short-delivery",$F33="Damaged goods"),AND($C33&lt;&gt;"",$D33&lt;&gt;"",$D33-$C33&gt;30)),OR(UPPER($E33)="Y",UPPER($E33)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F33="shortfall",$F33="damaged-goods",$F33="Shortfall / short-delivery",$F33="Damaged goods"),AND($C33&lt;&gt;"",$D33&lt;&gt;"",$D33-$C33&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I33="missing proof","Await line-level proof from the retailer.",IF($I33="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I33="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N33">
+        <f>IF($F33="","",IF(AND(AND(OR($F33="shortfall",$F33="damaged-goods",$F33="Shortfall / short-delivery",$F33="Damaged goods"),AND($C33&lt;&gt;"",$D33&lt;&gt;"",$D33-$C33&gt;30)),OR(UPPER($E33)="Y",UPPER($E33)="YES")),"High",IF(OR($I33="Code risk",$H33&gt;=5000),"High",IF(OR($I33="missing proof",$H33&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2282,33 +2448,38 @@
           <t/>
         </is>
       </c>
-      <c r="G34" s="3">
+      <c r="G34" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H34" s="3">
         <v>0</v>
       </c>
-      <c r="H34">
-        <f>IF($E34="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E34,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I34" s="2">
-        <f>IF($E34="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E34,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I34">
+        <f>IF($F34="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F34,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F34,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J34" s="2">
-        <f>IF($E34="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E34,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F34="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F34,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F34,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K34" s="2">
-        <f>IF($E34="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E34,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F34="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F34,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F34,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L34" s="2">
-        <f>IF(AND(OR($E34="shortfall",$E34="damaged-goods"),$C34&lt;&gt;"",$D34&lt;&gt;"",$D34-$C34&gt;30),"Claim raised more than 30 days after delivery.",IF($H34="missing proof","Await line-level proof from the retailer.",IF($H34="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H34="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M34">
-        <f>IF($E34="","",IF(AND(OR($E34="shortfall",$E34="damaged-goods"),$C34&lt;&gt;"",$D34&lt;&gt;"",$D34-$C34&gt;30),"High",IF(OR($H34="Code risk",$G34&gt;=5000),"High",IF(OR($H34="missing proof",$G34&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F34="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F34,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F34,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M34" s="2">
+        <f>IF(AND(AND(OR($F34="shortfall",$F34="damaged-goods",$F34="Shortfall / short-delivery",$F34="Damaged goods"),AND($C34&lt;&gt;"",$D34&lt;&gt;"",$D34-$C34&gt;30)),OR(UPPER($E34)="Y",UPPER($E34)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F34="shortfall",$F34="damaged-goods",$F34="Shortfall / short-delivery",$F34="Damaged goods"),AND($C34&lt;&gt;"",$D34&lt;&gt;"",$D34-$C34&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I34="missing proof","Await line-level proof from the retailer.",IF($I34="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I34="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N34">
+        <f>IF($F34="","",IF(AND(AND(OR($F34="shortfall",$F34="damaged-goods",$F34="Shortfall / short-delivery",$F34="Damaged goods"),AND($C34&lt;&gt;"",$D34&lt;&gt;"",$D34-$C34&gt;30)),OR(UPPER($E34)="Y",UPPER($E34)="YES")),"High",IF(OR($I34="Code risk",$H34&gt;=5000),"High",IF(OR($I34="missing proof",$H34&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2345,33 +2516,38 @@
           <t/>
         </is>
       </c>
-      <c r="G35" s="3">
+      <c r="G35" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H35" s="3">
         <v>0</v>
       </c>
-      <c r="H35">
-        <f>IF($E35="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E35,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I35" s="2">
-        <f>IF($E35="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E35,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I35">
+        <f>IF($F35="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F35,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F35,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J35" s="2">
-        <f>IF($E35="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E35,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F35="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F35,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F35,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K35" s="2">
-        <f>IF($E35="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E35,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F35="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F35,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F35,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L35" s="2">
-        <f>IF(AND(OR($E35="shortfall",$E35="damaged-goods"),$C35&lt;&gt;"",$D35&lt;&gt;"",$D35-$C35&gt;30),"Claim raised more than 30 days after delivery.",IF($H35="missing proof","Await line-level proof from the retailer.",IF($H35="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H35="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M35">
-        <f>IF($E35="","",IF(AND(OR($E35="shortfall",$E35="damaged-goods"),$C35&lt;&gt;"",$D35&lt;&gt;"",$D35-$C35&gt;30),"High",IF(OR($H35="Code risk",$G35&gt;=5000),"High",IF(OR($H35="missing proof",$G35&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F35="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F35,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F35,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M35" s="2">
+        <f>IF(AND(AND(OR($F35="shortfall",$F35="damaged-goods",$F35="Shortfall / short-delivery",$F35="Damaged goods"),AND($C35&lt;&gt;"",$D35&lt;&gt;"",$D35-$C35&gt;30)),OR(UPPER($E35)="Y",UPPER($E35)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F35="shortfall",$F35="damaged-goods",$F35="Shortfall / short-delivery",$F35="Damaged goods"),AND($C35&lt;&gt;"",$D35&lt;&gt;"",$D35-$C35&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I35="missing proof","Await line-level proof from the retailer.",IF($I35="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I35="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N35">
+        <f>IF($F35="","",IF(AND(AND(OR($F35="shortfall",$F35="damaged-goods",$F35="Shortfall / short-delivery",$F35="Damaged goods"),AND($C35&lt;&gt;"",$D35&lt;&gt;"",$D35-$C35&gt;30)),OR(UPPER($E35)="Y",UPPER($E35)="YES")),"High",IF(OR($I35="Code risk",$H35&gt;=5000),"High",IF(OR($I35="missing proof",$H35&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2408,33 +2584,38 @@
           <t/>
         </is>
       </c>
-      <c r="G36" s="3">
+      <c r="G36" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H36" s="3">
         <v>0</v>
       </c>
-      <c r="H36">
-        <f>IF($E36="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E36,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I36" s="2">
-        <f>IF($E36="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E36,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I36">
+        <f>IF($F36="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F36,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F36,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J36" s="2">
-        <f>IF($E36="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E36,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F36="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F36,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F36,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K36" s="2">
-        <f>IF($E36="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E36,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F36="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F36,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F36,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L36" s="2">
-        <f>IF(AND(OR($E36="shortfall",$E36="damaged-goods"),$C36&lt;&gt;"",$D36&lt;&gt;"",$D36-$C36&gt;30),"Claim raised more than 30 days after delivery.",IF($H36="missing proof","Await line-level proof from the retailer.",IF($H36="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H36="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M36">
-        <f>IF($E36="","",IF(AND(OR($E36="shortfall",$E36="damaged-goods"),$C36&lt;&gt;"",$D36&lt;&gt;"",$D36-$C36&gt;30),"High",IF(OR($H36="Code risk",$G36&gt;=5000),"High",IF(OR($H36="missing proof",$G36&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F36="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F36,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F36,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M36" s="2">
+        <f>IF(AND(AND(OR($F36="shortfall",$F36="damaged-goods",$F36="Shortfall / short-delivery",$F36="Damaged goods"),AND($C36&lt;&gt;"",$D36&lt;&gt;"",$D36-$C36&gt;30)),OR(UPPER($E36)="Y",UPPER($E36)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F36="shortfall",$F36="damaged-goods",$F36="Shortfall / short-delivery",$F36="Damaged goods"),AND($C36&lt;&gt;"",$D36&lt;&gt;"",$D36-$C36&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I36="missing proof","Await line-level proof from the retailer.",IF($I36="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I36="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N36">
+        <f>IF($F36="","",IF(AND(AND(OR($F36="shortfall",$F36="damaged-goods",$F36="Shortfall / short-delivery",$F36="Damaged goods"),AND($C36&lt;&gt;"",$D36&lt;&gt;"",$D36-$C36&gt;30)),OR(UPPER($E36)="Y",UPPER($E36)="YES")),"High",IF(OR($I36="Code risk",$H36&gt;=5000),"High",IF(OR($I36="missing proof",$H36&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2471,33 +2652,38 @@
           <t/>
         </is>
       </c>
-      <c r="G37" s="3">
+      <c r="G37" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H37" s="3">
         <v>0</v>
       </c>
-      <c r="H37">
-        <f>IF($E37="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E37,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I37" s="2">
-        <f>IF($E37="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E37,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I37">
+        <f>IF($F37="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F37,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F37,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J37" s="2">
-        <f>IF($E37="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E37,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F37="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F37,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F37,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K37" s="2">
-        <f>IF($E37="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E37,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F37="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F37,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F37,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L37" s="2">
-        <f>IF(AND(OR($E37="shortfall",$E37="damaged-goods"),$C37&lt;&gt;"",$D37&lt;&gt;"",$D37-$C37&gt;30),"Claim raised more than 30 days after delivery.",IF($H37="missing proof","Await line-level proof from the retailer.",IF($H37="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H37="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M37">
-        <f>IF($E37="","",IF(AND(OR($E37="shortfall",$E37="damaged-goods"),$C37&lt;&gt;"",$D37&lt;&gt;"",$D37-$C37&gt;30),"High",IF(OR($H37="Code risk",$G37&gt;=5000),"High",IF(OR($H37="missing proof",$G37&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F37="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F37,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F37,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M37" s="2">
+        <f>IF(AND(AND(OR($F37="shortfall",$F37="damaged-goods",$F37="Shortfall / short-delivery",$F37="Damaged goods"),AND($C37&lt;&gt;"",$D37&lt;&gt;"",$D37-$C37&gt;30)),OR(UPPER($E37)="Y",UPPER($E37)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F37="shortfall",$F37="damaged-goods",$F37="Shortfall / short-delivery",$F37="Damaged goods"),AND($C37&lt;&gt;"",$D37&lt;&gt;"",$D37-$C37&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I37="missing proof","Await line-level proof from the retailer.",IF($I37="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I37="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N37">
+        <f>IF($F37="","",IF(AND(AND(OR($F37="shortfall",$F37="damaged-goods",$F37="Shortfall / short-delivery",$F37="Damaged goods"),AND($C37&lt;&gt;"",$D37&lt;&gt;"",$D37-$C37&gt;30)),OR(UPPER($E37)="Y",UPPER($E37)="YES")),"High",IF(OR($I37="Code risk",$H37&gt;=5000),"High",IF(OR($I37="missing proof",$H37&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2534,33 +2720,38 @@
           <t/>
         </is>
       </c>
-      <c r="G38" s="3">
+      <c r="G38" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H38" s="3">
         <v>0</v>
       </c>
-      <c r="H38">
-        <f>IF($E38="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E38,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I38" s="2">
-        <f>IF($E38="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E38,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I38">
+        <f>IF($F38="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F38,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F38,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J38" s="2">
-        <f>IF($E38="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E38,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F38="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F38,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F38,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K38" s="2">
-        <f>IF($E38="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E38,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F38="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F38,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F38,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L38" s="2">
-        <f>IF(AND(OR($E38="shortfall",$E38="damaged-goods"),$C38&lt;&gt;"",$D38&lt;&gt;"",$D38-$C38&gt;30),"Claim raised more than 30 days after delivery.",IF($H38="missing proof","Await line-level proof from the retailer.",IF($H38="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H38="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M38">
-        <f>IF($E38="","",IF(AND(OR($E38="shortfall",$E38="damaged-goods"),$C38&lt;&gt;"",$D38&lt;&gt;"",$D38-$C38&gt;30),"High",IF(OR($H38="Code risk",$G38&gt;=5000),"High",IF(OR($H38="missing proof",$G38&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F38="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F38,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F38,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M38" s="2">
+        <f>IF(AND(AND(OR($F38="shortfall",$F38="damaged-goods",$F38="Shortfall / short-delivery",$F38="Damaged goods"),AND($C38&lt;&gt;"",$D38&lt;&gt;"",$D38-$C38&gt;30)),OR(UPPER($E38)="Y",UPPER($E38)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F38="shortfall",$F38="damaged-goods",$F38="Shortfall / short-delivery",$F38="Damaged goods"),AND($C38&lt;&gt;"",$D38&lt;&gt;"",$D38-$C38&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I38="missing proof","Await line-level proof from the retailer.",IF($I38="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I38="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N38">
+        <f>IF($F38="","",IF(AND(AND(OR($F38="shortfall",$F38="damaged-goods",$F38="Shortfall / short-delivery",$F38="Damaged goods"),AND($C38&lt;&gt;"",$D38&lt;&gt;"",$D38-$C38&gt;30)),OR(UPPER($E38)="Y",UPPER($E38)="YES")),"High",IF(OR($I38="Code risk",$H38&gt;=5000),"High",IF(OR($I38="missing proof",$H38&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2597,33 +2788,38 @@
           <t/>
         </is>
       </c>
-      <c r="G39" s="3">
+      <c r="G39" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H39" s="3">
         <v>0</v>
       </c>
-      <c r="H39">
-        <f>IF($E39="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E39,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I39" s="2">
-        <f>IF($E39="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E39,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I39">
+        <f>IF($F39="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F39,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F39,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J39" s="2">
-        <f>IF($E39="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E39,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F39="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F39,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F39,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K39" s="2">
-        <f>IF($E39="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E39,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F39="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F39,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F39,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L39" s="2">
-        <f>IF(AND(OR($E39="shortfall",$E39="damaged-goods"),$C39&lt;&gt;"",$D39&lt;&gt;"",$D39-$C39&gt;30),"Claim raised more than 30 days after delivery.",IF($H39="missing proof","Await line-level proof from the retailer.",IF($H39="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H39="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M39">
-        <f>IF($E39="","",IF(AND(OR($E39="shortfall",$E39="damaged-goods"),$C39&lt;&gt;"",$D39&lt;&gt;"",$D39-$C39&gt;30),"High",IF(OR($H39="Code risk",$G39&gt;=5000),"High",IF(OR($H39="missing proof",$G39&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F39="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F39,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F39,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M39" s="2">
+        <f>IF(AND(AND(OR($F39="shortfall",$F39="damaged-goods",$F39="Shortfall / short-delivery",$F39="Damaged goods"),AND($C39&lt;&gt;"",$D39&lt;&gt;"",$D39-$C39&gt;30)),OR(UPPER($E39)="Y",UPPER($E39)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F39="shortfall",$F39="damaged-goods",$F39="Shortfall / short-delivery",$F39="Damaged goods"),AND($C39&lt;&gt;"",$D39&lt;&gt;"",$D39-$C39&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I39="missing proof","Await line-level proof from the retailer.",IF($I39="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I39="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N39">
+        <f>IF($F39="","",IF(AND(AND(OR($F39="shortfall",$F39="damaged-goods",$F39="Shortfall / short-delivery",$F39="Damaged goods"),AND($C39&lt;&gt;"",$D39&lt;&gt;"",$D39-$C39&gt;30)),OR(UPPER($E39)="Y",UPPER($E39)="YES")),"High",IF(OR($I39="Code risk",$H39&gt;=5000),"High",IF(OR($I39="missing proof",$H39&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2660,33 +2856,38 @@
           <t/>
         </is>
       </c>
-      <c r="G40" s="3">
+      <c r="G40" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H40" s="3">
         <v>0</v>
       </c>
-      <c r="H40">
-        <f>IF($E40="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E40,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I40" s="2">
-        <f>IF($E40="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E40,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I40">
+        <f>IF($F40="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F40,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F40,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J40" s="2">
-        <f>IF($E40="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E40,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F40="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F40,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F40,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K40" s="2">
-        <f>IF($E40="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E40,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F40="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F40,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F40,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L40" s="2">
-        <f>IF(AND(OR($E40="shortfall",$E40="damaged-goods"),$C40&lt;&gt;"",$D40&lt;&gt;"",$D40-$C40&gt;30),"Claim raised more than 30 days after delivery.",IF($H40="missing proof","Await line-level proof from the retailer.",IF($H40="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H40="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M40">
-        <f>IF($E40="","",IF(AND(OR($E40="shortfall",$E40="damaged-goods"),$C40&lt;&gt;"",$D40&lt;&gt;"",$D40-$C40&gt;30),"High",IF(OR($H40="Code risk",$G40&gt;=5000),"High",IF(OR($H40="missing proof",$G40&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F40="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F40,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F40,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M40" s="2">
+        <f>IF(AND(AND(OR($F40="shortfall",$F40="damaged-goods",$F40="Shortfall / short-delivery",$F40="Damaged goods"),AND($C40&lt;&gt;"",$D40&lt;&gt;"",$D40-$C40&gt;30)),OR(UPPER($E40)="Y",UPPER($E40)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F40="shortfall",$F40="damaged-goods",$F40="Shortfall / short-delivery",$F40="Damaged goods"),AND($C40&lt;&gt;"",$D40&lt;&gt;"",$D40-$C40&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I40="missing proof","Await line-level proof from the retailer.",IF($I40="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I40="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N40">
+        <f>IF($F40="","",IF(AND(AND(OR($F40="shortfall",$F40="damaged-goods",$F40="Shortfall / short-delivery",$F40="Damaged goods"),AND($C40&lt;&gt;"",$D40&lt;&gt;"",$D40-$C40&gt;30)),OR(UPPER($E40)="Y",UPPER($E40)="YES")),"High",IF(OR($I40="Code risk",$H40&gt;=5000),"High",IF(OR($I40="missing proof",$H40&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O40" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2723,33 +2924,38 @@
           <t/>
         </is>
       </c>
-      <c r="G41" s="3">
+      <c r="G41" t="inlineStr" s="2">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H41" s="3">
         <v>0</v>
       </c>
-      <c r="H41">
-        <f>IF($E41="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,MATCH($E41,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
-      </c>
-      <c r="I41" s="2">
-        <f>IF($E41="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,MATCH($E41,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+      <c r="I41">
+        <f>IF($F41="","",INDEX('Deduction Type Matrix'!$C$2:$C$17,IFERROR(MATCH($F41,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F41,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="J41" s="2">
-        <f>IF($E41="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,MATCH($E41,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F41="","",INDEX('Deduction Type Matrix'!$D$2:$D$17,IFERROR(MATCH($F41,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F41,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="K41" s="2">
-        <f>IF($E41="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,MATCH($E41,'Deduction Type Matrix'!$A$2:$A$17,0)))</f>
+        <f>IF($F41="","",INDEX('Deduction Type Matrix'!$E$2:$E$17,IFERROR(MATCH($F41,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F41,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
       </c>
       <c r="L41" s="2">
-        <f>IF(AND(OR($E41="shortfall",$E41="damaged-goods"),$C41&lt;&gt;"",$D41&lt;&gt;"",$D41-$C41&gt;30),"Claim raised more than 30 days after delivery.",IF($H41="missing proof","Await line-level proof from the retailer.",IF($H41="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($H41="worth challenging","Reconcile this line against prior credits, timing, and support.",""))))</f>
-      </c>
-      <c r="M41">
-        <f>IF($E41="","",IF(AND(OR($E41="shortfall",$E41="damaged-goods"),$C41&lt;&gt;"",$D41&lt;&gt;"",$D41-$C41&gt;30),"High",IF(OR($H41="Code risk",$G41&gt;=5000),"High",IF(OR($H41="missing proof",$G41&gt;=1000),"Medium","Low"))))</f>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <f>IF($F41="","",INDEX('Deduction Type Matrix'!$F$2:$F$17,IFERROR(MATCH($F41,'Deduction Type Matrix'!$A$2:$A$17,0),MATCH($F41,'Deduction Type Matrix'!$B$2:$B$17,0))))</f>
+      </c>
+      <c r="M41" s="2">
+        <f>IF(AND(AND(OR($F41="shortfall",$F41="damaged-goods",$F41="Shortfall / short-delivery",$F41="Damaged goods"),AND($C41&lt;&gt;"",$D41&lt;&gt;"",$D41-$C41&gt;30)),OR(UPPER($E41)="Y",UPPER($E41)="YES")),"Fresh produce claim raised more than 30 days after delivery.",IF(AND(OR($F41="shortfall",$F41="damaged-goods",$F41="Shortfall / short-delivery",$F41="Damaged goods"),AND($C41&lt;&gt;"",$D41&lt;&gt;"",$D41-$C41&gt;30)),"If this line is fresh produce, check why the claim was raised more than 30 days after delivery.",IF($I41="missing proof","Await line-level proof from the retailer.",IF($I41="Code risk","Check Code coverage, agreement basis, and retailer conditions.",IF($I41="worth challenging","Reconcile this line against prior credits, timing, and support.","")))))</f>
+      </c>
+      <c r="N41">
+        <f>IF($F41="","",IF(AND(AND(OR($F41="shortfall",$F41="damaged-goods",$F41="Shortfall / short-delivery",$F41="Damaged goods"),AND($C41&lt;&gt;"",$D41&lt;&gt;"",$D41-$C41&gt;30)),OR(UPPER($E41)="Y",UPPER($E41)="YES")),"High",IF(OR($I41="Code risk",$H41&gt;=5000),"High",IF(OR($I41="missing proof",$H41&gt;=1000),"Medium","Low"))))</f>
       </c>
       <c r="O41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -3054,7 +3260,7 @@
       </c>
       <c r="E6" t="inlineStr" s="2">
         <is>
-          <t>Check the Code's 30-day cap on retailer-raised shortfall claims.</t>
+          <t>For fresh produce, check the Code's 30-day cap on retailer-raised shortfall claims.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="2">
@@ -3064,7 +3270,7 @@
       </c>
       <c r="G6" t="inlineStr" s="2">
         <is>
-          <t>The Code caps retailer-raised shortfall claims at no later than 30 days after delivery where the Code applies.</t>
+          <t>For fresh produce, the Code caps retailer-raised shortfall claims at no later than 30 days after delivery where the Code applies.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -3074,7 +3280,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>claimRaisedWithinDays</t>
+          <t>freshProduceClaimRaisedWithinDays</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -3106,7 +3312,7 @@
       </c>
       <c r="E7" t="inlineStr" s="2">
         <is>
-          <t>Check the Code's 30-day cap on retailer-raised damage claims.</t>
+          <t>For fresh produce, check the Code's 30-day cap on retailer-raised damage claims.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="2">
@@ -3116,7 +3322,7 @@
       </c>
       <c r="G7" t="inlineStr" s="2">
         <is>
-          <t>The Code caps retailer-raised damage claims at no later than 30 days after delivery where the Code applies.</t>
+          <t>For fresh produce, the Code caps retailer-raised damage claims at no later than 30 days after delivery where the Code applies.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -3126,7 +3332,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>claimRaisedWithinDays</t>
+          <t>freshProduceClaimRaisedWithinDays</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -3686,7 +3892,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>SUMIF('Claim Ledger'!$H$2:$H$41,A2,'Claim Ledger'!$G$2:$G$41)</f>
+        <f>SUMIF('Claim Ledger'!$I$2:$I$41,A2,'Claim Ledger'!$H$2:$H$41)</f>
       </c>
     </row>
     <row r="3">
@@ -3696,7 +3902,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>SUMIF('Claim Ledger'!$H$2:$H$41,A3,'Claim Ledger'!$G$2:$G$41)</f>
+        <f>SUMIF('Claim Ledger'!$I$2:$I$41,A3,'Claim Ledger'!$H$2:$H$41)</f>
       </c>
     </row>
     <row r="4">
@@ -3706,7 +3912,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>SUMIF('Claim Ledger'!$H$2:$H$41,A4,'Claim Ledger'!$G$2:$G$41)</f>
+        <f>SUMIF('Claim Ledger'!$I$2:$I$41,A4,'Claim Ledger'!$H$2:$H$41)</f>
       </c>
     </row>
     <row r="5">
@@ -3716,7 +3922,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>SUMIF('Claim Ledger'!$H$2:$H$41,A5,'Claim Ledger'!$G$2:$G$41)</f>
+        <f>SUMIF('Claim Ledger'!$I$2:$I$41,A5,'Claim Ledger'!$H$2:$H$41)</f>
       </c>
     </row>
     <row r="7">

</xml_diff>